<commit_message>
update redis model excel
</commit_message>
<xml_diff>
--- a/redis_forum_modele.xlsx
+++ b/redis_forum_modele.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mathis Francoise\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mathis Francoise\Desktop\cours25-26\redis\forumInsta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6355CE41-C5FA-4D68-A401-D52DD0C18E8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C70D365-6E02-46B9-AC2F-2E54F25EC01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="74">
   <si>
     <t>Question métier</t>
   </si>
@@ -38,28 +38,13 @@
     <t>Vérifier les identifiants à la connexion</t>
   </si>
   <si>
-    <t>GET user:email:{email} → récupère l'ID
-HGETALL user:{id} → récupère hash+salt</t>
-  </si>
-  <si>
     <t>Élevée</t>
   </si>
   <si>
-    <t>Récupérer le profil de l'utilisateur connecté</t>
-  </si>
-  <si>
-    <t>HGETALL user:{id}</t>
-  </si>
-  <si>
     <t>Hash</t>
   </si>
   <si>
     <t>Créer un nouvel utilisateur</t>
-  </si>
-  <si>
-    <t>INCR user:next_id
-HSET user:{id} ...
-SET user:email:{email} {id}</t>
   </si>
   <si>
     <t>Faible</t>
@@ -73,12 +58,6 @@
   <si>
     <t>LRANGE forums 0 -1 → liste d'IDs
 HGETALL forum:{id} → détail de chaque forum</t>
-  </si>
-  <si>
-    <t>Récupérer le détail d'un forum</t>
-  </si>
-  <si>
-    <t>HGETALL forum:{id}</t>
   </si>
   <si>
     <t>Créer un nouveau forum</t>
@@ -101,176 +80,185 @@
     <t>HINCRBY forum:{id} visits 1</t>
   </si>
   <si>
-    <t>Posts</t>
-  </si>
-  <si>
-    <t>Lister les posts d'un forum</t>
+    <t>Moyenne</t>
+  </si>
+  <si>
+    <t>Likes</t>
+  </si>
+  <si>
+    <t>Set</t>
+  </si>
+  <si>
+    <t>Voir le nombre de likes d'un post</t>
+  </si>
+  <si>
+    <t>Vérifier si l'utilisateur a liké un post</t>
+  </si>
+  <si>
+    <t>Clé</t>
+  </si>
+  <si>
+    <t>Contenu / Champs</t>
+  </si>
+  <si>
+    <t>Opérations principales</t>
+  </si>
+  <si>
+    <t>user:next_id</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>Compteur auto-increment des users</t>
+  </si>
+  <si>
+    <t>INCR user:next_id</t>
+  </si>
+  <si>
+    <t>forum:next_id</t>
+  </si>
+  <si>
+    <t>Compteur auto-increment des forums</t>
+  </si>
+  <si>
+    <t>INCR forum:next_id</t>
+  </si>
+  <si>
+    <t>user:{id}</t>
+  </si>
+  <si>
+    <t>HSET / HGETALL / HGET</t>
+  </si>
+  <si>
+    <t>ID de l'utilisateur (index par email)</t>
+  </si>
+  <si>
+    <t>SET / GET</t>
+  </si>
+  <si>
+    <t>forum:{id}</t>
+  </si>
+  <si>
+    <t>HSET / HGETALL / HINCRBY</t>
+  </si>
+  <si>
+    <t>forums</t>
+  </si>
+  <si>
+    <t>List</t>
+  </si>
+  <si>
+    <t>Liste de tous les IDs de forums</t>
+  </si>
+  <si>
+    <t>LPUSH / LRANGE</t>
+  </si>
+  <si>
+    <t>HSET / HGETALL</t>
+  </si>
+  <si>
+    <t>SADD / SREM / SCARD / SISMEMBER</t>
+  </si>
+  <si>
+    <t>Compteurs</t>
+  </si>
+  <si>
+    <t>Utilisateurs</t>
+  </si>
+  <si>
+    <t>Criticité</t>
+  </si>
+  <si>
+    <t>Basse</t>
+  </si>
+  <si>
+    <t>Lister les messages d'un forum</t>
+  </si>
+  <si>
+    <t>Créer un message dans un forum</t>
+  </si>
+  <si>
+    <t>Liker un message (un like par utilisateur)</t>
+  </si>
+  <si>
+    <t>Retirer son like d'un message</t>
+  </si>
+  <si>
+    <t>SADD message:{id}:likes {user_id}</t>
+  </si>
+  <si>
+    <t>SREM message:{id}:likes {user_id}</t>
+  </si>
+  <si>
+    <t>SCARD message:{id}:likes</t>
+  </si>
+  <si>
+    <t>SISMEMBER message:{id}:likes {user_id}</t>
   </si>
   <si>
     <t>LRANGE forum:{id}:posts 0 -1 → liste d'IDs
-HGETALL post:{id} → détail de chaque post</t>
-  </si>
-  <si>
-    <t>Récupérer le détail d'un post</t>
-  </si>
-  <si>
-    <t>HGETALL post:{id}</t>
-  </si>
-  <si>
-    <t>Créer un post dans un forum</t>
-  </si>
-  <si>
-    <t>INCR post:next_id
-HSET post:{id} ...
-LPUSH forum:{forum_id}:posts {id}</t>
-  </si>
-  <si>
-    <t>Moyenne</t>
-  </si>
-  <si>
-    <t>Likes</t>
-  </si>
-  <si>
-    <t>Liker un post (un like par utilisateur)</t>
-  </si>
-  <si>
-    <t>SADD post:{id}:likes {user_id}</t>
-  </si>
-  <si>
-    <t>Set</t>
-  </si>
-  <si>
-    <t>Retirer son like d'un post</t>
-  </si>
-  <si>
-    <t>SREM post:{id}:likes {user_id}</t>
-  </si>
-  <si>
-    <t>Voir le nombre de likes d'un post</t>
-  </si>
-  <si>
-    <t>SCARD post:{id}:likes</t>
-  </si>
-  <si>
-    <t>Vérifier si l'utilisateur a liké un post</t>
-  </si>
-  <si>
-    <t>SISMEMBER post:{id}:likes {user_id}</t>
-  </si>
-  <si>
-    <t>Clé</t>
-  </si>
-  <si>
-    <t>Contenu / Champs</t>
-  </si>
-  <si>
-    <t>Opérations principales</t>
-  </si>
-  <si>
-    <t>user:next_id</t>
-  </si>
-  <si>
-    <t>String</t>
-  </si>
-  <si>
-    <t>Compteur auto-increment des users</t>
-  </si>
-  <si>
-    <t>INCR user:next_id</t>
-  </si>
-  <si>
-    <t>forum:next_id</t>
-  </si>
-  <si>
-    <t>Compteur auto-increment des forums</t>
-  </si>
-  <si>
-    <t>INCR forum:next_id</t>
-  </si>
-  <si>
-    <t>post:next_id</t>
-  </si>
-  <si>
-    <t>Compteur auto-increment des posts</t>
-  </si>
-  <si>
-    <t>INCR post:next_id</t>
-  </si>
-  <si>
-    <t>user:{id}</t>
-  </si>
-  <si>
-    <t>id, username, email, password, created_at</t>
-  </si>
-  <si>
-    <t>HSET / HGETALL / HGET</t>
-  </si>
-  <si>
-    <t>user:email:{email}</t>
-  </si>
-  <si>
-    <t>ID de l'utilisateur (index par email)</t>
-  </si>
-  <si>
-    <t>SET / GET</t>
-  </si>
-  <si>
-    <t>forum:{id}</t>
-  </si>
-  <si>
-    <t>id, title, description, created_by, created_at, visits</t>
-  </si>
-  <si>
-    <t>HSET / HGETALL / HINCRBY</t>
-  </si>
-  <si>
-    <t>forums</t>
-  </si>
-  <si>
-    <t>List</t>
-  </si>
-  <si>
-    <t>Liste de tous les IDs de forums</t>
-  </si>
-  <si>
-    <t>LPUSH / LRANGE</t>
-  </si>
-  <si>
-    <t>post:{id}</t>
-  </si>
-  <si>
-    <t>id, title, content, forum_id, created_by, created_at</t>
-  </si>
-  <si>
-    <t>HSET / HGETALL</t>
-  </si>
-  <si>
-    <t>forum:{id}:posts</t>
-  </si>
-  <si>
-    <t>Liste des IDs de posts d'un forum</t>
-  </si>
-  <si>
-    <t>post:{id}:likes</t>
-  </si>
-  <si>
-    <t>Ensemble des user_id ayant liké le post</t>
-  </si>
-  <si>
-    <t>SADD / SREM / SCARD / SISMEMBER</t>
-  </si>
-  <si>
-    <t>Compteurs</t>
-  </si>
-  <si>
-    <t>Utilisateurs</t>
+HGETALL message:{id} → détail de chaque message</t>
+  </si>
+  <si>
+    <t>INCR message:next_id
+HSET message:{id} ...
+LPUSH forum:{forum_id}:messages {id}</t>
+  </si>
+  <si>
+    <t>id, username, password</t>
+  </si>
+  <si>
+    <t>GET user:username:{username} → récupère l'ID
+HGETALL user:{id} → récupère hash+salt</t>
+  </si>
+  <si>
+    <t>INCR user:next_id
+HSET user:{id} ...
+SET user:username:{username} {id}</t>
+  </si>
+  <si>
+    <t>user:username:{username}</t>
+  </si>
+  <si>
+    <t>id, title, creator, visits</t>
+  </si>
+  <si>
+    <t>id, content, forum_id, creator, created_at</t>
+  </si>
+  <si>
+    <t>message:next_id</t>
+  </si>
+  <si>
+    <t>Compteur auto-increment des messages</t>
+  </si>
+  <si>
+    <t>INCR message:next_id</t>
+  </si>
+  <si>
+    <t>message:{id}</t>
+  </si>
+  <si>
+    <t>forum:{id}:messages</t>
+  </si>
+  <si>
+    <t>Liste des IDs de messages d'un forum</t>
+  </si>
+  <si>
+    <t>message:{id}:likes</t>
+  </si>
+  <si>
+    <t>Ensemble des user_id ayant liké le message</t>
+  </si>
+  <si>
+    <t>Messages</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -297,6 +285,31 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -340,29 +353,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -665,16 +690,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42" style="2" customWidth="1"/>
     <col min="2" max="2" width="46" style="2" customWidth="1"/>
     <col min="3" max="3" width="12" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.7265625" style="2"/>
+    <col min="4" max="4" width="11.08984375" style="13" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,170 +710,176 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="D1" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D2" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D3" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="C6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="C7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="3" t="s">
+      <c r="D9" s="11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="B12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>34</v>
+      <c r="B13" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -868,196 +900,196 @@
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="9" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="7" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
     </row>
     <row r="3" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="7" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" s="9" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
     </row>
     <row r="7" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>57</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" s="9" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="7" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
     </row>
     <row r="10" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="9" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="7" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="9" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="7" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
     </row>
     <row r="16" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>